<commit_message>
Add T-score (50 + 10 z) as second normalisation in scoring model and brief
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkWScMhuRmEB4zppSmB7Ri
</commit_message>
<xml_diff>
--- a/WT26-27/Country Scoring Model Template.xlsx
+++ b/WT26-27/Country Scoring Model Template.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicators" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Normalised" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Z-scores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="T-scores" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scores" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubrics" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,9 +173,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -643,7 +640,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Each indicator is rescaled to 0 to 100 across the six countries (min-max, direction respected). The score of a country is the weighted sum of its indicator scores. The Z-scores sheet shows a second normalisation.</t>
+          <t>Each indicator is rescaled to 0 to 100 across the six countries (min-max, direction respected). The score of a country is the weighted sum of its indicator scores. The T-scores sheet shows a second normalisation (50 + 10 x z-score; 50 = average of the six countries).</t>
         </is>
       </c>
     </row>
@@ -3360,14 +3357,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Z-scores (centred and scaled, direction respected)</t>
+          <t>T-scores (z-scores rescaled: 50 + 10 x z, direction respected)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Value minus mean, divided by the standard deviation of the six countries. Positive = better than average.</t>
+          <t>z = (value - mean) / standard deviation of the six countries; T = 50 + 10 x z. 50 = average of the six countries, 60 = one standard deviation better. Not capped at 0 or 100.</t>
         </is>
       </c>
     </row>
@@ -3422,28 +3419,28 @@
         <f>Indicators!C4</f>
         <v/>
       </c>
-      <c r="C4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!D5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
-        <v/>
-      </c>
-      <c r="D4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!G5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
-        <v/>
-      </c>
-      <c r="E4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!J5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
-        <v/>
-      </c>
-      <c r="F4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!M5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
-        <v/>
-      </c>
-      <c r="G4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!P5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
-        <v/>
-      </c>
-      <c r="H4" s="19">
-        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!S5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)))</f>
+      <c r="C4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!D5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!G5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!J5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!M5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!P5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H4" s="13">
+        <f>IF(COUNT(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)&lt;6,"",IF(STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)=0,"",IF(Data!$C5="Lower is better",-1,1)*(Data!S5-AVERAGE(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5))/STDEVP(Data!D5,Data!G5,Data!J5,Data!M5,Data!P5,Data!S5)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3456,28 +3453,28 @@
         <f>Indicators!C5</f>
         <v/>
       </c>
-      <c r="C5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!D6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
-        <v/>
-      </c>
-      <c r="D5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!G6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
-        <v/>
-      </c>
-      <c r="E5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!J6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
-        <v/>
-      </c>
-      <c r="F5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!M6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
-        <v/>
-      </c>
-      <c r="G5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!P6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
-        <v/>
-      </c>
-      <c r="H5" s="19">
-        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!S6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)))</f>
+      <c r="C5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!D6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!G6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!J6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!M6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!P6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H5" s="13">
+        <f>IF(COUNT(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)&lt;6,"",IF(STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)=0,"",IF(Data!$C6="Lower is better",-1,1)*(Data!S6-AVERAGE(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6))/STDEVP(Data!D6,Data!G6,Data!J6,Data!M6,Data!P6,Data!S6)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3490,28 +3487,28 @@
         <f>Indicators!C6</f>
         <v/>
       </c>
-      <c r="C6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!D7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
-        <v/>
-      </c>
-      <c r="D6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!G7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
-        <v/>
-      </c>
-      <c r="E6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!J7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
-        <v/>
-      </c>
-      <c r="F6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!M7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
-        <v/>
-      </c>
-      <c r="G6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!P7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
-        <v/>
-      </c>
-      <c r="H6" s="19">
-        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!S7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)))</f>
+      <c r="C6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!D7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!G7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!J7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!M7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!P7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H6" s="13">
+        <f>IF(COUNT(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)&lt;6,"",IF(STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)=0,"",IF(Data!$C7="Lower is better",-1,1)*(Data!S7-AVERAGE(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7))/STDEVP(Data!D7,Data!G7,Data!J7,Data!M7,Data!P7,Data!S7)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3524,28 +3521,28 @@
         <f>Indicators!C7</f>
         <v/>
       </c>
-      <c r="C7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!D8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
-        <v/>
-      </c>
-      <c r="D7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!G8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
-        <v/>
-      </c>
-      <c r="E7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!J8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
-        <v/>
-      </c>
-      <c r="F7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!M8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
-        <v/>
-      </c>
-      <c r="G7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!P8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
-        <v/>
-      </c>
-      <c r="H7" s="19">
-        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!S8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)))</f>
+      <c r="C7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!D8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!G8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!J8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!M8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!P8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>IF(COUNT(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)&lt;6,"",IF(STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)=0,"",IF(Data!$C8="Lower is better",-1,1)*(Data!S8-AVERAGE(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8))/STDEVP(Data!D8,Data!G8,Data!J8,Data!M8,Data!P8,Data!S8)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3558,28 +3555,28 @@
         <f>Indicators!C8</f>
         <v/>
       </c>
-      <c r="C8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!D9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
-        <v/>
-      </c>
-      <c r="D8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!G9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
-        <v/>
-      </c>
-      <c r="E8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!J9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
-        <v/>
-      </c>
-      <c r="F8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!M9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
-        <v/>
-      </c>
-      <c r="G8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!P9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
-        <v/>
-      </c>
-      <c r="H8" s="19">
-        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!S9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)))</f>
+      <c r="C8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!D9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!G9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!J9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!M9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!P9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H8" s="13">
+        <f>IF(COUNT(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)&lt;6,"",IF(STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)=0,"",IF(Data!$C9="Lower is better",-1,1)*(Data!S9-AVERAGE(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9))/STDEVP(Data!D9,Data!G9,Data!J9,Data!M9,Data!P9,Data!S9)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3592,28 +3589,28 @@
         <f>Indicators!C9</f>
         <v/>
       </c>
-      <c r="C9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!D10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
-        <v/>
-      </c>
-      <c r="D9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!G10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
-        <v/>
-      </c>
-      <c r="E9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!J10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
-        <v/>
-      </c>
-      <c r="F9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!M10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
-        <v/>
-      </c>
-      <c r="G9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!P10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
-        <v/>
-      </c>
-      <c r="H9" s="19">
-        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!S10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)))</f>
+      <c r="C9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!D10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!G10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!J10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!M10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!P10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H9" s="13">
+        <f>IF(COUNT(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)&lt;6,"",IF(STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)=0,"",IF(Data!$C10="Lower is better",-1,1)*(Data!S10-AVERAGE(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10))/STDEVP(Data!D10,Data!G10,Data!J10,Data!M10,Data!P10,Data!S10)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3626,28 +3623,28 @@
         <f>Indicators!C10</f>
         <v/>
       </c>
-      <c r="C10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!D11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!G11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
-        <v/>
-      </c>
-      <c r="E10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!J11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
-        <v/>
-      </c>
-      <c r="F10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!M11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
-        <v/>
-      </c>
-      <c r="G10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!P11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
-        <v/>
-      </c>
-      <c r="H10" s="19">
-        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!S11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)))</f>
+      <c r="C10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!D11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!G11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!J11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!M11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!P11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H10" s="13">
+        <f>IF(COUNT(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)&lt;6,"",IF(STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)=0,"",IF(Data!$C11="Lower is better",-1,1)*(Data!S11-AVERAGE(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11))/STDEVP(Data!D11,Data!G11,Data!J11,Data!M11,Data!P11,Data!S11)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3660,28 +3657,28 @@
         <f>Indicators!C11</f>
         <v/>
       </c>
-      <c r="C11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!D12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
-        <v/>
-      </c>
-      <c r="D11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!G12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
-        <v/>
-      </c>
-      <c r="E11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!J12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
-        <v/>
-      </c>
-      <c r="F11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!M12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
-        <v/>
-      </c>
-      <c r="G11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!P12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
-        <v/>
-      </c>
-      <c r="H11" s="19">
-        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!S12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)))</f>
+      <c r="C11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!D12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!G12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!J12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!M12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!P12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H11" s="13">
+        <f>IF(COUNT(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)&lt;6,"",IF(STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)=0,"",IF(Data!$C12="Lower is better",-1,1)*(Data!S12-AVERAGE(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12))/STDEVP(Data!D12,Data!G12,Data!J12,Data!M12,Data!P12,Data!S12)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3694,28 +3691,28 @@
         <f>Indicators!C12</f>
         <v/>
       </c>
-      <c r="C12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!D13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
-        <v/>
-      </c>
-      <c r="D12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!G13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
-        <v/>
-      </c>
-      <c r="E12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!J13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
-        <v/>
-      </c>
-      <c r="F12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!M13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
-        <v/>
-      </c>
-      <c r="G12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!P13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
-        <v/>
-      </c>
-      <c r="H12" s="19">
-        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!S13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)))</f>
+      <c r="C12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!D13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!G13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!J13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!M13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!P13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H12" s="13">
+        <f>IF(COUNT(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)&lt;6,"",IF(STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)=0,"",IF(Data!$C13="Lower is better",-1,1)*(Data!S13-AVERAGE(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13))/STDEVP(Data!D13,Data!G13,Data!J13,Data!M13,Data!P13,Data!S13)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3728,28 +3725,28 @@
         <f>Indicators!C13</f>
         <v/>
       </c>
-      <c r="C13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!D14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
-        <v/>
-      </c>
-      <c r="D13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!G14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
-        <v/>
-      </c>
-      <c r="E13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!J14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
-        <v/>
-      </c>
-      <c r="F13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!M14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
-        <v/>
-      </c>
-      <c r="G13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!P14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
-        <v/>
-      </c>
-      <c r="H13" s="19">
-        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!S14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)))</f>
+      <c r="C13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!D14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!G14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!J14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!M14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!P14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H13" s="13">
+        <f>IF(COUNT(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)&lt;6,"",IF(STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)=0,"",IF(Data!$C14="Lower is better",-1,1)*(Data!S14-AVERAGE(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14))/STDEVP(Data!D14,Data!G14,Data!J14,Data!M14,Data!P14,Data!S14)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3762,28 +3759,28 @@
         <f>Indicators!C14</f>
         <v/>
       </c>
-      <c r="C14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!D15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
-        <v/>
-      </c>
-      <c r="D14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!G15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
-        <v/>
-      </c>
-      <c r="E14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!J15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
-        <v/>
-      </c>
-      <c r="F14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!M15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
-        <v/>
-      </c>
-      <c r="G14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!P15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
-        <v/>
-      </c>
-      <c r="H14" s="19">
-        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!S15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)))</f>
+      <c r="C14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!D15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!G15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!J15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!M15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!P15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H14" s="13">
+        <f>IF(COUNT(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)&lt;6,"",IF(STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)=0,"",IF(Data!$C15="Lower is better",-1,1)*(Data!S15-AVERAGE(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15))/STDEVP(Data!D15,Data!G15,Data!J15,Data!M15,Data!P15,Data!S15)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3796,28 +3793,28 @@
         <f>Indicators!C15</f>
         <v/>
       </c>
-      <c r="C15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!D16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
-        <v/>
-      </c>
-      <c r="D15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!G16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
-        <v/>
-      </c>
-      <c r="E15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!J16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
-        <v/>
-      </c>
-      <c r="F15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!M16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
-        <v/>
-      </c>
-      <c r="G15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!P16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
-        <v/>
-      </c>
-      <c r="H15" s="19">
-        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!S16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)))</f>
+      <c r="C15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!D16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!G16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!J16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!M16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!P16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H15" s="13">
+        <f>IF(COUNT(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)&lt;6,"",IF(STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)=0,"",IF(Data!$C16="Lower is better",-1,1)*(Data!S16-AVERAGE(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16))/STDEVP(Data!D16,Data!G16,Data!J16,Data!M16,Data!P16,Data!S16)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3830,28 +3827,28 @@
         <f>Indicators!C16</f>
         <v/>
       </c>
-      <c r="C16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!D17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
-        <v/>
-      </c>
-      <c r="D16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!G17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
-        <v/>
-      </c>
-      <c r="E16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!J17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
-        <v/>
-      </c>
-      <c r="F16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!M17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
-        <v/>
-      </c>
-      <c r="G16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!P17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
-        <v/>
-      </c>
-      <c r="H16" s="19">
-        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!S17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)))</f>
+      <c r="C16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!D17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!G17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!J17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!M17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!P17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H16" s="13">
+        <f>IF(COUNT(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)&lt;6,"",IF(STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)=0,"",IF(Data!$C17="Lower is better",-1,1)*(Data!S17-AVERAGE(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17))/STDEVP(Data!D17,Data!G17,Data!J17,Data!M17,Data!P17,Data!S17)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3864,28 +3861,28 @@
         <f>Indicators!C17</f>
         <v/>
       </c>
-      <c r="C17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!D18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
-        <v/>
-      </c>
-      <c r="D17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!G18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
-        <v/>
-      </c>
-      <c r="E17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!J18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
-        <v/>
-      </c>
-      <c r="F17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!M18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
-        <v/>
-      </c>
-      <c r="G17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!P18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
-        <v/>
-      </c>
-      <c r="H17" s="19">
-        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!S18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)))</f>
+      <c r="C17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!D18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
+        <v/>
+      </c>
+      <c r="D17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!G18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
+        <v/>
+      </c>
+      <c r="E17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!J18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
+        <v/>
+      </c>
+      <c r="F17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!M18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
+        <v/>
+      </c>
+      <c r="G17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!P18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
+        <v/>
+      </c>
+      <c r="H17" s="13">
+        <f>IF(COUNT(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)&lt;6,"",IF(STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)=0,"",IF(Data!$C18="Lower is better",-1,1)*(Data!S18-AVERAGE(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18))/STDEVP(Data!D18,Data!G18,Data!J18,Data!M18,Data!P18,Data!S18)*10+50))</f>
         <v/>
       </c>
     </row>
@@ -3927,7 +3924,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>A. Weighted score (0 to 100, min-max)</t>
         </is>
@@ -4128,7 +4125,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>B. Rank (1 = best)</t>
         </is>
@@ -4358,7 +4355,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>C. Baseline score by PESTEL dimension (average of the indicator scores)</t>
         </is>
@@ -4588,9 +4585,9 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="inlineStr">
-        <is>
-          <t>D. Baseline weights with z-scores (second normalisation)</t>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>D. Baseline weights with T-scores (second normalisation)</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4599,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Weighted z-score</t>
+          <t>Weighted T-score</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -4617,8 +4614,8 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B32" s="19">
-        <f>IF(COUNT('Z-scores'!C4:C17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!C4:C17)/100)</f>
+      <c r="B32" s="13">
+        <f>IF(COUNT('T-scores'!C4:C17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!C4:C17)/100)</f>
         <v/>
       </c>
       <c r="C32" s="8">
@@ -4632,8 +4629,8 @@
           <t>Brazil</t>
         </is>
       </c>
-      <c r="B33" s="19">
-        <f>IF(COUNT('Z-scores'!D4:D17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!D4:D17)/100)</f>
+      <c r="B33" s="13">
+        <f>IF(COUNT('T-scores'!D4:D17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!D4:D17)/100)</f>
         <v/>
       </c>
       <c r="C33" s="8">
@@ -4647,8 +4644,8 @@
           <t>Chile</t>
         </is>
       </c>
-      <c r="B34" s="19">
-        <f>IF(COUNT('Z-scores'!E4:E17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!E4:E17)/100)</f>
+      <c r="B34" s="13">
+        <f>IF(COUNT('T-scores'!E4:E17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!E4:E17)/100)</f>
         <v/>
       </c>
       <c r="C34" s="8">
@@ -4662,8 +4659,8 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B35" s="19">
-        <f>IF(COUNT('Z-scores'!F4:F17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!F4:F17)/100)</f>
+      <c r="B35" s="13">
+        <f>IF(COUNT('T-scores'!F4:F17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!F4:F17)/100)</f>
         <v/>
       </c>
       <c r="C35" s="8">
@@ -4677,8 +4674,8 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="B36" s="19">
-        <f>IF(COUNT('Z-scores'!G4:G17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!G4:G17)/100)</f>
+      <c r="B36" s="13">
+        <f>IF(COUNT('T-scores'!G4:G17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!G4:G17)/100)</f>
         <v/>
       </c>
       <c r="C36" s="8">
@@ -4692,8 +4689,8 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B37" s="19">
-        <f>IF(COUNT('Z-scores'!H4:H17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'Z-scores'!H4:H17)/100)</f>
+      <c r="B37" s="13">
+        <f>IF(COUNT('T-scores'!H4:H17)&lt;14,"incomplete",SUMPRODUCT(Weights!C17:C30,'T-scores'!H4:H17)/100)</f>
         <v/>
       </c>
       <c r="C37" s="8">

</xml_diff>

<commit_message>
Scoring model: students enter numbers only, everything else automatic and locked; brief updated
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkWScMhuRmEB4zppSmB7Ri
</commit_message>
<xml_diff>
--- a/WT26-27/Country Scoring Model Template.xlsx
+++ b/WT26-27/Country Scoring Model Template.xlsx
@@ -168,11 +168,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -551,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -604,7 +606,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Only on the Data sheet, only in the yellow cells of your own country: value, year and source (name and link). Do not type in other groups' columns. Never type over a grey or white cell: they contain formulas.</t>
+          <t>Only the numbers: on the Data sheet, in the yellow cells of your own country, enter the value of each indicator (rubric indicators: a whole number from 1 to 5). Next to each value, note the year and the source link for documentation. Everything else (normalisation, weights, scores, ranks, robustness) is calculated by the sheet. Only the yellow cells can be edited; the other sheets are locked. Do not type in other groups' columns.</t>
         </is>
       </c>
     </row>
@@ -635,64 +637,77 @@
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>How scores are calculated</t>
+          <t>Normalisation is automatic</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Each indicator is rescaled to 0 to 100 across the six countries (min-max, direction respected). The score of a country is the weighted sum of its indicator scores. The T-scores sheet shows a second normalisation (50 + 10 x z-score; 50 = average of the six countries).</t>
+          <t>You do not normalise anything yourself. As soon as the data of all six countries are entered, the sheet rescales every indicator across the six countries: the Normalised sheet gives min-max scores from 0 to 100 and the T-scores sheet gives 50 + 10 x z-score (50 = average of the six countries). The direction of each indicator (higher or lower is better) is applied automatically.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Robustness</t>
+          <t>How scores are calculated</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>The Scores sheet recalculates the ranking with four alternative weight sets. Use it for Step 7 of the student brief.</t>
+          <t>The score of a country is the weighted sum of its normalised indicator scores (sheet Scores). All results update by themselves when a value changes.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="40" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Colour code</t>
+          <t>Robustness</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Yellow with blue text: input. Grey: fixed by the instructor. White or light grey with black text: formula.</t>
+          <t>The Scores sheet recalculates the ranking with four alternative weight sets. Use it for Step 7 of the student brief.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="40" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Quality rules</t>
+          <t>Colour code</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Use the latest year available. Use the unit given. Record the year and a source link for every value. Qualitative scores use the rubrics on the Rubrics sheet; write the reason in the source cell. A country with a missing value shows "incomplete" instead of a score.</t>
+          <t>Yellow with blue text: input. Grey: fixed by the instructor. White or light grey with black text: formula.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
+          <t>Quality rules</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Use the latest year available. Use the unit given. Record the year and a source link for every value. Qualitative scores use the rubrics on the Rubrics sheet; write the reason in the source cell. A country with a missing value shows "incomplete" instead of a score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>arne.floh@wu.ac.at</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1446,6 +1461,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A12:G13"/>
   </mergeCells>
@@ -2117,6 +2133,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2761,6 +2778,7 @@
       <c r="U18" s="18" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="6">
     <mergeCell ref="M3:O3"/>
     <mergeCell ref="D3:F3"/>
@@ -3331,6 +3349,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3887,6 +3906,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4699,6 +4719,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <conditionalFormatting sqref="B14:F19">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>B14=1</formula>
@@ -4874,6 +4895,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scoring model: indicator list is an example until instructor selection
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RkWScMhuRmEB4zppSmB7Ri
</commit_message>
<xml_diff>
--- a/WT26-27/Country Scoring Model Template.xlsx
+++ b/WT26-27/Country Scoring Model Template.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>The 45 indicators are grouped by the six PESTEL dimensions (Political, Economic, Social, Technological, Environmental, Legal). Julius Meinl's six dimensions are shown as a second label.</t>
+          <t>The 45 indicators (selected by the instructor from the proposals of all groups; the list in this template is an example until then) are grouped by the six PESTEL dimensions (Political, Economic, Social, Technological, Environmental, Legal). Julius Meinl's six dimensions are shown as a second label.</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Proposed by the instructor from the group shortlists. Same for all groups.</t>
+          <t>EXAMPLE LIST. After the PESTEL search (45 criteria per group, due session 3) the instructor merges the proposals and replaces this list with the final selection: 5 political, 10 economic, 10 social, 10 technological, 5 environmental, 5 legal. Same for all groups.</t>
         </is>
       </c>
     </row>

</xml_diff>